<commit_message>
fix: evitar Bad Request por header de cookie sobredimensionado en carga/actualizacion masiva
TempData usaba el proveedor de cookies por defecto para guardar la
previsualizacion completa del Excel (JSON de todas las filas), lo que
generaba cookies de varios KB que Apache (proxy reverso) rechazaba al
confirmar con "Size of a request header field exceeds server limit".
Se cambia a AddSessionStateTempDataProvider() para que TempData use la
sesion del servidor en vez de cookies.

De paso se regeneran las plantillas de carga/actualizacion masiva de
equipos: seguian ofreciendo "Telefono" en el desplegable de tipo de
equipo, cuando el tipo por defecto se renombro a "Celular" (5985928).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/wwwroot/plantilla_equipos.xlsx
+++ b/wwwroot/plantilla_equipos.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipos" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Referencia" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Equipos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Referencia" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -828,8 +828,8 @@
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="B5:B24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Tipo inválido" error="Valor no válido. Use: Laptop, Teléfono, Tablet u Otro" type="list">
-      <formula1>"Laptop,Teléfono,Tablet,Otro"</formula1>
+    <dataValidation sqref="B5:B24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Tipo inválido" error="Valor no válido. Use: Laptop, Celular, Tablet u Otro" type="list">
+      <formula1>"Laptop,Celular,Tablet,Otro"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -866,7 +866,7 @@
     <row r="3">
       <c r="A3" s="11" t="inlineStr">
         <is>
-          <t>Teléfono</t>
+          <t>Celular</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: soportar IMEI en carga masiva de equipos nuevos (celulares)
La plantilla y el controlador de Carga Masiva no tenían columna de
IMEI, a diferencia del alta individual donde es obligatorio para tipo
Celular. Al insertar una columna manualmente para poder cargarlo, se
corrían todas las columnas siguientes (Modelo terminaba leyendose
como Serie, etc).

Se agrega la columna IMEI a la plantilla (wwwroot/plantilla_equipos.xlsx,
generada con el nuevo generar_plantilla_carga.py), se lee y persiste en
el controlador, se valida como obligatoria para tipo Celular (igual que
en el alta individual) y se muestra en la previsualización para poder
verificar que las columnas se leyeron bien antes de confirmar.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/wwwroot/plantilla_equipos.xlsx
+++ b/wwwroot/plantilla_equipos.xlsx
@@ -154,9 +154,7 @@
     <xf numFmtId="164" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -534,10 +532,11 @@
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -583,20 +582,25 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
+          <t>IMEI</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
           <t>Accesorios</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>Costo</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>FechaCompra</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>FechaGarantia</t>
         </is>
@@ -609,9 +613,10 @@
       <c r="D5" s="4" t="n"/>
       <c r="E5" s="4" t="n"/>
       <c r="F5" s="4" t="n"/>
-      <c r="G5" s="5" t="n"/>
-      <c r="H5" s="6" t="n"/>
+      <c r="G5" s="4" t="n"/>
+      <c r="H5" s="5" t="n"/>
       <c r="I5" s="6" t="n"/>
+      <c r="J5" s="6" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="7" t="n"/>
@@ -620,9 +625,10 @@
       <c r="D6" s="7" t="n"/>
       <c r="E6" s="7" t="n"/>
       <c r="F6" s="7" t="n"/>
-      <c r="G6" s="8" t="n"/>
-      <c r="H6" s="9" t="n"/>
+      <c r="G6" s="7" t="n"/>
+      <c r="H6" s="8" t="n"/>
       <c r="I6" s="9" t="n"/>
+      <c r="J6" s="9" t="n"/>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="4" t="n"/>
@@ -631,9 +637,10 @@
       <c r="D7" s="4" t="n"/>
       <c r="E7" s="4" t="n"/>
       <c r="F7" s="4" t="n"/>
-      <c r="G7" s="5" t="n"/>
-      <c r="H7" s="6" t="n"/>
+      <c r="G7" s="4" t="n"/>
+      <c r="H7" s="5" t="n"/>
       <c r="I7" s="6" t="n"/>
+      <c r="J7" s="6" t="n"/>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="7" t="n"/>
@@ -642,9 +649,10 @@
       <c r="D8" s="7" t="n"/>
       <c r="E8" s="7" t="n"/>
       <c r="F8" s="7" t="n"/>
-      <c r="G8" s="8" t="n"/>
-      <c r="H8" s="9" t="n"/>
+      <c r="G8" s="7" t="n"/>
+      <c r="H8" s="8" t="n"/>
       <c r="I8" s="9" t="n"/>
+      <c r="J8" s="9" t="n"/>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="4" t="n"/>
@@ -653,9 +661,10 @@
       <c r="D9" s="4" t="n"/>
       <c r="E9" s="4" t="n"/>
       <c r="F9" s="4" t="n"/>
-      <c r="G9" s="5" t="n"/>
-      <c r="H9" s="6" t="n"/>
+      <c r="G9" s="4" t="n"/>
+      <c r="H9" s="5" t="n"/>
       <c r="I9" s="6" t="n"/>
+      <c r="J9" s="6" t="n"/>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="7" t="n"/>
@@ -664,9 +673,10 @@
       <c r="D10" s="7" t="n"/>
       <c r="E10" s="7" t="n"/>
       <c r="F10" s="7" t="n"/>
-      <c r="G10" s="8" t="n"/>
-      <c r="H10" s="9" t="n"/>
+      <c r="G10" s="7" t="n"/>
+      <c r="H10" s="8" t="n"/>
       <c r="I10" s="9" t="n"/>
+      <c r="J10" s="9" t="n"/>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="4" t="n"/>
@@ -675,9 +685,10 @@
       <c r="D11" s="4" t="n"/>
       <c r="E11" s="4" t="n"/>
       <c r="F11" s="4" t="n"/>
-      <c r="G11" s="5" t="n"/>
-      <c r="H11" s="6" t="n"/>
+      <c r="G11" s="4" t="n"/>
+      <c r="H11" s="5" t="n"/>
       <c r="I11" s="6" t="n"/>
+      <c r="J11" s="6" t="n"/>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="7" t="n"/>
@@ -686,9 +697,10 @@
       <c r="D12" s="7" t="n"/>
       <c r="E12" s="7" t="n"/>
       <c r="F12" s="7" t="n"/>
-      <c r="G12" s="8" t="n"/>
-      <c r="H12" s="9" t="n"/>
+      <c r="G12" s="7" t="n"/>
+      <c r="H12" s="8" t="n"/>
       <c r="I12" s="9" t="n"/>
+      <c r="J12" s="9" t="n"/>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="4" t="n"/>
@@ -697,9 +709,10 @@
       <c r="D13" s="4" t="n"/>
       <c r="E13" s="4" t="n"/>
       <c r="F13" s="4" t="n"/>
-      <c r="G13" s="5" t="n"/>
-      <c r="H13" s="6" t="n"/>
+      <c r="G13" s="4" t="n"/>
+      <c r="H13" s="5" t="n"/>
       <c r="I13" s="6" t="n"/>
+      <c r="J13" s="6" t="n"/>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="7" t="n"/>
@@ -708,9 +721,10 @@
       <c r="D14" s="7" t="n"/>
       <c r="E14" s="7" t="n"/>
       <c r="F14" s="7" t="n"/>
-      <c r="G14" s="8" t="n"/>
-      <c r="H14" s="9" t="n"/>
+      <c r="G14" s="7" t="n"/>
+      <c r="H14" s="8" t="n"/>
       <c r="I14" s="9" t="n"/>
+      <c r="J14" s="9" t="n"/>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="4" t="n"/>
@@ -719,9 +733,10 @@
       <c r="D15" s="4" t="n"/>
       <c r="E15" s="4" t="n"/>
       <c r="F15" s="4" t="n"/>
-      <c r="G15" s="5" t="n"/>
-      <c r="H15" s="6" t="n"/>
+      <c r="G15" s="4" t="n"/>
+      <c r="H15" s="5" t="n"/>
       <c r="I15" s="6" t="n"/>
+      <c r="J15" s="6" t="n"/>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="7" t="n"/>
@@ -730,9 +745,10 @@
       <c r="D16" s="7" t="n"/>
       <c r="E16" s="7" t="n"/>
       <c r="F16" s="7" t="n"/>
-      <c r="G16" s="8" t="n"/>
-      <c r="H16" s="9" t="n"/>
+      <c r="G16" s="7" t="n"/>
+      <c r="H16" s="8" t="n"/>
       <c r="I16" s="9" t="n"/>
+      <c r="J16" s="9" t="n"/>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="4" t="n"/>
@@ -741,9 +757,10 @@
       <c r="D17" s="4" t="n"/>
       <c r="E17" s="4" t="n"/>
       <c r="F17" s="4" t="n"/>
-      <c r="G17" s="5" t="n"/>
-      <c r="H17" s="6" t="n"/>
+      <c r="G17" s="4" t="n"/>
+      <c r="H17" s="5" t="n"/>
       <c r="I17" s="6" t="n"/>
+      <c r="J17" s="6" t="n"/>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="7" t="n"/>
@@ -752,9 +769,10 @@
       <c r="D18" s="7" t="n"/>
       <c r="E18" s="7" t="n"/>
       <c r="F18" s="7" t="n"/>
-      <c r="G18" s="8" t="n"/>
-      <c r="H18" s="9" t="n"/>
+      <c r="G18" s="7" t="n"/>
+      <c r="H18" s="8" t="n"/>
       <c r="I18" s="9" t="n"/>
+      <c r="J18" s="9" t="n"/>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="4" t="n"/>
@@ -763,9 +781,10 @@
       <c r="D19" s="4" t="n"/>
       <c r="E19" s="4" t="n"/>
       <c r="F19" s="4" t="n"/>
-      <c r="G19" s="5" t="n"/>
-      <c r="H19" s="6" t="n"/>
+      <c r="G19" s="4" t="n"/>
+      <c r="H19" s="5" t="n"/>
       <c r="I19" s="6" t="n"/>
+      <c r="J19" s="6" t="n"/>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="7" t="n"/>
@@ -774,9 +793,10 @@
       <c r="D20" s="7" t="n"/>
       <c r="E20" s="7" t="n"/>
       <c r="F20" s="7" t="n"/>
-      <c r="G20" s="8" t="n"/>
-      <c r="H20" s="9" t="n"/>
+      <c r="G20" s="7" t="n"/>
+      <c r="H20" s="8" t="n"/>
       <c r="I20" s="9" t="n"/>
+      <c r="J20" s="9" t="n"/>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="4" t="n"/>
@@ -785,9 +805,10 @@
       <c r="D21" s="4" t="n"/>
       <c r="E21" s="4" t="n"/>
       <c r="F21" s="4" t="n"/>
-      <c r="G21" s="5" t="n"/>
-      <c r="H21" s="6" t="n"/>
+      <c r="G21" s="4" t="n"/>
+      <c r="H21" s="5" t="n"/>
       <c r="I21" s="6" t="n"/>
+      <c r="J21" s="6" t="n"/>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="7" t="n"/>
@@ -796,9 +817,10 @@
       <c r="D22" s="7" t="n"/>
       <c r="E22" s="7" t="n"/>
       <c r="F22" s="7" t="n"/>
-      <c r="G22" s="8" t="n"/>
-      <c r="H22" s="9" t="n"/>
+      <c r="G22" s="7" t="n"/>
+      <c r="H22" s="8" t="n"/>
       <c r="I22" s="9" t="n"/>
+      <c r="J22" s="9" t="n"/>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="4" t="n"/>
@@ -807,9 +829,10 @@
       <c r="D23" s="4" t="n"/>
       <c r="E23" s="4" t="n"/>
       <c r="F23" s="4" t="n"/>
-      <c r="G23" s="5" t="n"/>
-      <c r="H23" s="6" t="n"/>
+      <c r="G23" s="4" t="n"/>
+      <c r="H23" s="5" t="n"/>
       <c r="I23" s="6" t="n"/>
+      <c r="J23" s="6" t="n"/>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="7" t="n"/>
@@ -818,9 +841,10 @@
       <c r="D24" s="7" t="n"/>
       <c r="E24" s="7" t="n"/>
       <c r="F24" s="7" t="n"/>
-      <c r="G24" s="8" t="n"/>
-      <c r="H24" s="9" t="n"/>
+      <c r="G24" s="7" t="n"/>
+      <c r="H24" s="8" t="n"/>
       <c r="I24" s="9" t="n"/>
+      <c r="J24" s="9" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -828,7 +852,7 @@
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="B5:B24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Tipo inválido" error="Valor no válido. Use: Laptop, Celular, Tablet u Otro" type="list">
+    <dataValidation sqref="B5:B24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Tipo inválido" error="Valor no válido. Use: Laptop, Celular, Tablet u Otro" type="list">
       <formula1>"Laptop,Celular,Tablet,Otro"</formula1>
     </dataValidation>
   </dataValidations>
@@ -842,7 +866,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -927,9 +951,6 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:B1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>